<commit_message>
update data to admission students
</commit_message>
<xml_diff>
--- a/public/template/plantilla_alumnos.xlsx
+++ b/public/template/plantilla_alumnos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\constancias\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zero/Desktop/UPRIT/certificate-api/public/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C907ABCE-284B-44AE-B7D0-3E134680AC6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC27B7D-877D-2040-9068-9FB2F5B64EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DD4E6A56-8447-4AEF-B429-CAC84584CCD9}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{DD4E6A56-8447-4AEF-B429-CAC84584CCD9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>FULL_NAME</t>
   </si>
@@ -42,43 +42,22 @@
     <t>DNI</t>
   </si>
   <si>
-    <t>STUDENT_CODE</t>
-  </si>
-  <si>
-    <t>PROGRAM</t>
-  </si>
-  <si>
-    <t>ISSUE_DATE</t>
-  </si>
-  <si>
-    <t>MODALITY</t>
-  </si>
-  <si>
-    <t>START_SEMESTER</t>
-  </si>
-  <si>
-    <t>START_DATE</t>
-  </si>
-  <si>
-    <t>CERTIFICATE_CODE</t>
-  </si>
-  <si>
-    <t>FACULTY</t>
-  </si>
-  <si>
-    <t>GRADUATION_SEMESTER</t>
-  </si>
-  <si>
-    <t>GRADUATION_DATE</t>
-  </si>
-  <si>
-    <t>CREDITS</t>
-  </si>
-  <si>
-    <t>ACADEMIC_CYCLE</t>
-  </si>
-  <si>
-    <t>CURRENT_SEMESTER</t>
+    <t>NOMBRE</t>
+  </si>
+  <si>
+    <t>APELLIDO</t>
+  </si>
+  <si>
+    <t>TIPO PROGRAMA</t>
+  </si>
+  <si>
+    <t>PROGRAMA</t>
+  </si>
+  <si>
+    <t>PERIODO</t>
+  </si>
+  <si>
+    <t>CORREO</t>
   </si>
 </sst>
 </file>
@@ -97,6 +76,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -121,9 +101,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -143,9 +122,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -183,7 +162,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -289,7 +268,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -431,7 +410,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -439,22 +418,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{035A6447-A205-48F5-B27A-D913AE63024F}">
-  <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -468,37 +444,19 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>